<commit_message>
Stage 8 review fixes: G-013
</commit_message>
<xml_diff>
--- a/output/heldback_firm_G/OsterquillData/Studies/OT-25-S0229/Protocol/Amendments/VP28_Protocol_Hold_102725.xlsx
+++ b/output/heldback_firm_G/OsterquillData/Studies/OT-25-S0229/Protocol/Amendments/VP28_Protocol_Hold_102725.xlsx
@@ -152,7 +152,7 @@
         <t>Upper dose cell is still open. Nothing goes to Valquessia until Naomi has seen the revised rationale.</t>
       </text>
     </comment>
-    <comment ref="B9" authorId="1" shapeId="0">
+    <comment ref="B7" authorId="1" shapeId="0">
       <text>
         <t>Dosing schedule for the recovery arm not drafted. Rachel to take it on once the vehicle is signed off.</t>
       </text>
@@ -568,7 +568,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Pre-dosing formulation hold: new vehicle to be qualified before dosing starts</t>
+          <t>Pre-dosing formulation hold: new formulation to be qualified before dosing starts</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -739,7 +739,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Unchanged from the draft protocol</t>
+          <t>Control vehicle to be aligned with the qualified formulation; amendment approval pending</t>
         </is>
       </c>
     </row>
@@ -783,6 +783,14 @@
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Animal numbers and sex split: to be confirmed at the study start meeting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Pre-dosing hold: no animal dosing results or tolerated-dose conclusion recorded.</t>
         </is>
       </c>
     </row>

</xml_diff>